<commit_message>
chore(results): regenerate all Excel workbooks with latest canonical 5D benchmark results
</commit_message>
<xml_diff>
--- a/results/calibration_results_m3_llava.xlsx
+++ b/results/calibration_results_m3_llava.xlsx
@@ -1052,16 +1052,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0414273062484926</v>
+        <v>0.0391826856168453</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0501616478287627</v>
+        <v>0.0472977394363629</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.7529309596178897</v>
+        <v>0.7640758431031986</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.0922221920498468</v>
+        <v>0.091654400562028</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -1100,16 +1100,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0373331835484226</v>
+        <v>0.0366356788447157</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0404301009535699</v>
+        <v>0.0401177829367202</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.7599507888261687</v>
+        <v>0.7647271674627298</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.0912712100033132</v>
+        <v>0.0910499760159712</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -1396,16 +1396,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0234770833026795</v>
+        <v>0.0268204004991622</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0584313000951494</v>
+        <v>0.0465042852220081</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.7046290951075191</v>
+        <v>0.7025364410448838</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.1436529792216732</v>
+        <v>0.1446549727715895</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -1444,16 +1444,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0371789375207253</v>
+        <v>0.036756165053013</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.053045153375367</v>
+        <v>0.0482579440536738</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.7030054841968538</v>
+        <v>0.7048816568047337</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.1447752259739189</v>
+        <v>0.1445917528181202</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -1740,16 +1740,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0303326041698455</v>
+        <v>0.0293322855234146</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0582579566240311</v>
+        <v>0.0560587364435196</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.6422401198042224</v>
+        <v>0.6337478997735408</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.2068452232914008</v>
+        <v>0.2079118232056215</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -1788,16 +1788,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.043037573225953</v>
+        <v>0.0675958988634682</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.085196952952394</v>
+        <v>0.0682452025709889</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.6346245160347725</v>
+        <v>0.6287438819490101</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.2092699348741287</v>
+        <v>0.2107795645358461</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -2084,16 +2084,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0477382720708847</v>
+        <v>0.060169622041285</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0410459154844284</v>
+        <v>0.0587407152280211</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.84245826709062</v>
+        <v>0.8408684419713832</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.1593429496603514</v>
+        <v>0.1601246446390918</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -2132,16 +2132,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.05311773230252</v>
+        <v>0.0503419091019339</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0538658790639865</v>
+        <v>0.0612237164300177</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.8338135930047694</v>
+        <v>0.8337307896131425</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.1624713302642987</v>
+        <v>0.1626005650131539</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -2428,16 +2428,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0530126131051219</v>
+        <v>0.0620477101691067</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0655327024930156</v>
+        <v>0.0708762660212815</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.8329767295284536</v>
+        <v>0.8377038032210447</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.1643438469670865</v>
+        <v>0.1633380640559222</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -2476,16 +2476,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0672173624858665</v>
+        <v>0.0678958133778107</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0735274564543615</v>
+        <v>0.073954757100471</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.8356636977326632</v>
+        <v>0.8355807666152493</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.1638630026167679</v>
+        <v>0.1640010055809327</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -2772,16 +2772,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0693080826774239</v>
+        <v>0.0683666338324546</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0640767282024025</v>
+        <v>0.0787226635813713</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.794808201058201</v>
+        <v>0.7819822373393802</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.138849684087251</v>
+        <v>0.1438549670349855</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -2820,16 +2820,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0539624282673602</v>
+        <v>0.0457087304183394</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0872338009946871</v>
+        <v>0.0698432642811654</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.7684476568405141</v>
+        <v>0.7713293650793651</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.1421961134863753</v>
+        <v>0.1420311404618216</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -3116,16 +3116,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0697438307702541</v>
+        <v>0.0702362337708473</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0951195200383663</v>
+        <v>0.09526135188341139</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.6416087078051267</v>
+        <v>0.6452424406846545</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.2317422742093862</v>
+        <v>0.2308868159950006</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -3164,16 +3164,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.070485540669318</v>
+        <v>0.0576318766674033</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0776557364810911</v>
+        <v>0.113556592789863</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.6370953156086092</v>
+        <v>0.6371610845295055</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.2326304127804471</v>
+        <v>0.2321490955087143</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -3460,16 +3460,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0260600510798394</v>
+        <v>0.0341114686783403</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0303687149249017</v>
+        <v>0.0326657267417758</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.8366788766788767</v>
+        <v>0.8274969474969475</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.0678570668880064</v>
+        <v>0.06841858290559499</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -3508,16 +3508,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0353072762232562</v>
+        <v>0.0328300596575699</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.028573757152288</v>
+        <v>0.0203230087741482</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.8375579975579975</v>
+        <v>0.8360439560439561</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.0681968408259913</v>
+        <v>0.06834949014000891</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -3804,16 +3804,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0190104336244985</v>
+        <v>0.0203513838630169</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0311087451316416</v>
+        <v>0.0292766467407345</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.7303157093952074</v>
+        <v>0.7371624191707874</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.0411096069592869</v>
+        <v>0.0409190969283196</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -3852,16 +3852,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0204670697028163</v>
+        <v>0.020085814597341</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0265385653757316</v>
+        <v>0.0253431584352759</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.7384937238493723</v>
+        <v>0.7370673259794599</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.0417855434375025</v>
+        <v>0.041785784144644</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -4148,16 +4148,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.07970090188086031</v>
+        <v>0.0468183397948741</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0829537709206343</v>
+        <v>0.0447280292809009</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.6869093139023157</v>
+        <v>0.7004094221196163</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.2012851297457719</v>
+        <v>0.1985484469333324</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -4196,16 +4196,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0521689957563656</v>
+        <v>0.0592273545790596</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0670718376626256</v>
+        <v>0.0597775249170785</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.7035116513960031</v>
+        <v>0.7080748142269677</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.1950084866893705</v>
+        <v>0.1946969446585122</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -4492,16 +4492,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0002055465642479</v>
+        <v>0.0002762173963128</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0110544629067298</v>
+        <v>0.0102832866431563</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.595766129032258</v>
+        <v>0.6617943548387096</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.0079335527989073</v>
+        <v>0.007913245330409199</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -4540,16 +4540,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0005746748163085</v>
+        <v>0.0005804956777396</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0131362795449365</v>
+        <v>0.0131390633456571</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.4248991935483871</v>
+        <v>0.4223790322580645</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.0079429239996589</v>
+        <v>0.0079429398750417</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -4836,16 +4836,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0797823336652734</v>
+        <v>0.0564491748809814</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0845849592238664</v>
+        <v>0.1028657380830157</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.6426992314980524</v>
+        <v>0.6522791872828718</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.1909877173957252</v>
+        <v>0.1899148505707685</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -4884,16 +4884,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0088700498393788</v>
+        <v>0.008683075327286301</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.099317354764587</v>
+        <v>0.09944458685460961</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.5085798505105801</v>
+        <v>0.5206863880408463</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.1941779525474872</v>
+        <v>0.1942508168171545</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -5180,16 +5180,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.044602942764759</v>
+        <v>0.0409236796974873</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0661013222336769</v>
+        <v>0.0528613575816416</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.6893400716930129</v>
+        <v>0.6910834263775438</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.1855853661404867</v>
+        <v>0.1869267030177952</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -5228,16 +5228,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0517824057243972</v>
+        <v>0.057882151166305</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0454666756398896</v>
+        <v>0.0537903234560563</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.6906916612798966</v>
+        <v>0.6905545434957199</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.1855416536542819</v>
+        <v>0.1885566072289334</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
@@ -5524,16 +5524,16 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.0191789832455744</v>
+        <v>0.0169348890827508</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.0354046452214281</v>
+        <v>0.0364822698151286</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.641025641025641</v>
+        <v>0.6252465483234714</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0.020697718558281</v>
+        <v>0.0199436581497105</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
@@ -5572,16 +5572,16 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.0188953981072319</v>
+        <v>0.0195528363078007</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.0347526995121748</v>
+        <v>0.0345077535957687</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>0.6390532544378698</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.0208107188032083</v>
+        <v>0.0205869240392087</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">

</xml_diff>